<commit_message>
change .xslm files to .xslx file types, add additional raw data and ingestion processes to load_to _snowflake.py, new cleaning in EDA
</commit_message>
<xml_diff>
--- a/data/raw/timeliness/timeliness-medicaid-sept-2025.xlsx
+++ b/data/raw/timeliness/timeliness-medicaid-sept-2025.xlsx
@@ -1,19 +1,19 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28925"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10510"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="Z:\READ ONLY WEB FILES\Medicaid Timeliness\FY2025\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/jameslavin/Downloads/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{F04122B4-D8D6-4CD1-82BC-570F5907960D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A4C078BC-E95D-6E4B-A8A4-83865D23D404}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{F1717CFB-4D1D-4320-938C-407D063ABBEC}"/>
+    <workbookView xWindow="0" yWindow="600" windowWidth="23260" windowHeight="12460" xr2:uid="{F1717CFB-4D1D-4320-938C-407D063ABBEC}"/>
   </bookViews>
   <sheets>
-    <sheet name="Medcaid" sheetId="1" r:id="rId1"/>
+    <sheet name="Medicaid" sheetId="1" r:id="rId1"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -455,74 +455,74 @@
   <cellXfs count="30">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="49" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="49" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" indent="1"/>
+    </xf>
+    <xf numFmtId="10" fontId="4" fillId="0" borderId="9" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="4" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" indent="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="4" fillId="0" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" indent="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="4" fillId="0" borderId="17" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" indent="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="18" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" indent="1"/>
-    </xf>
-    <xf numFmtId="10" fontId="4" fillId="0" borderId="9" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="3" fontId="4" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" indent="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="3" fontId="4" fillId="0" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" indent="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="3" fontId="4" fillId="0" borderId="17" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" indent="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="18" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
@@ -865,718 +865,718 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{18352712-B40D-432C-A2CA-BDAF5177DA96}">
   <dimension ref="A1:T60"/>
-  <sheetFormatPr defaultRowHeight="16.2" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.625" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="9.3046875" customWidth="1"/>
-    <col min="2" max="2" width="8.61328125" customWidth="1"/>
-    <col min="3" max="4" width="7.69140625" customWidth="1"/>
-    <col min="6" max="6" width="9.3046875" customWidth="1"/>
-    <col min="7" max="7" width="7.921875" customWidth="1"/>
-    <col min="8" max="8" width="7.23046875" customWidth="1"/>
-    <col min="9" max="9" width="8.61328125" customWidth="1"/>
-    <col min="10" max="10" width="7.69140625" customWidth="1"/>
-    <col min="11" max="11" width="7.07421875" customWidth="1"/>
+    <col min="1" max="1" width="9.25" customWidth="1"/>
+    <col min="2" max="2" width="8.625" customWidth="1"/>
+    <col min="3" max="4" width="7.75" customWidth="1"/>
+    <col min="6" max="6" width="9.25" customWidth="1"/>
+    <col min="7" max="7" width="7.875" customWidth="1"/>
+    <col min="8" max="8" width="7.25" customWidth="1"/>
+    <col min="9" max="9" width="8.625" customWidth="1"/>
+    <col min="10" max="10" width="7.75" customWidth="1"/>
+    <col min="11" max="11" width="7.125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:20" ht="17.399999999999999" x14ac:dyDescent="0.3">
-      <c r="A1" s="1" t="s">
+    <row r="1" spans="1:20" ht="18" x14ac:dyDescent="0.2">
+      <c r="A1" s="22" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1"/>
-      <c r="C1" s="1"/>
-      <c r="D1" s="1"/>
-      <c r="E1" s="1"/>
-      <c r="F1" s="1"/>
-      <c r="G1" s="1"/>
-      <c r="H1" s="1"/>
-      <c r="I1" s="1"/>
-      <c r="J1" s="1"/>
-      <c r="K1" s="2"/>
-      <c r="L1" s="3"/>
-      <c r="M1" s="3"/>
-      <c r="N1" s="3"/>
-      <c r="O1" s="3"/>
-      <c r="P1" s="3"/>
-      <c r="Q1" s="3"/>
-      <c r="R1" s="3"/>
-      <c r="S1" s="3"/>
-      <c r="T1" s="3"/>
-    </row>
-    <row r="2" spans="1:20" ht="18.899999999999999" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A2" s="2"/>
-      <c r="B2" s="3"/>
-      <c r="C2" s="3"/>
-      <c r="D2" s="3"/>
-      <c r="E2" s="3"/>
-      <c r="F2" s="3"/>
-      <c r="G2" s="3"/>
-      <c r="H2" s="3"/>
-      <c r="I2" s="3"/>
-      <c r="J2" s="3"/>
-      <c r="K2" s="3"/>
-      <c r="L2" s="3"/>
-      <c r="M2" s="3"/>
-      <c r="N2" s="3"/>
-      <c r="O2" s="3"/>
-      <c r="P2" s="3"/>
-      <c r="Q2" s="3"/>
-      <c r="R2" s="3"/>
-      <c r="S2" s="3"/>
-      <c r="T2" s="3"/>
-    </row>
-    <row r="3" spans="1:20" ht="18" customHeight="1" thickTop="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="4" t="s">
+      <c r="B1" s="22"/>
+      <c r="C1" s="22"/>
+      <c r="D1" s="22"/>
+      <c r="E1" s="22"/>
+      <c r="F1" s="22"/>
+      <c r="G1" s="22"/>
+      <c r="H1" s="22"/>
+      <c r="I1" s="22"/>
+      <c r="J1" s="22"/>
+      <c r="K1" s="1"/>
+      <c r="L1" s="2"/>
+      <c r="M1" s="2"/>
+      <c r="N1" s="2"/>
+      <c r="O1" s="2"/>
+      <c r="P1" s="2"/>
+      <c r="Q1" s="2"/>
+      <c r="R1" s="2"/>
+      <c r="S1" s="2"/>
+      <c r="T1" s="2"/>
+    </row>
+    <row r="2" spans="1:20" ht="19" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A2" s="1"/>
+      <c r="B2" s="2"/>
+      <c r="C2" s="2"/>
+      <c r="D2" s="2"/>
+      <c r="E2" s="2"/>
+      <c r="F2" s="2"/>
+      <c r="G2" s="2"/>
+      <c r="H2" s="2"/>
+      <c r="I2" s="2"/>
+      <c r="J2" s="2"/>
+      <c r="K2" s="2"/>
+      <c r="L2" s="2"/>
+      <c r="M2" s="2"/>
+      <c r="N2" s="2"/>
+      <c r="O2" s="2"/>
+      <c r="P2" s="2"/>
+      <c r="Q2" s="2"/>
+      <c r="R2" s="2"/>
+      <c r="S2" s="2"/>
+      <c r="T2" s="2"/>
+    </row>
+    <row r="3" spans="1:20" ht="18" customHeight="1" thickTop="1" x14ac:dyDescent="0.2">
+      <c r="A3" s="23" t="s">
         <v>1</v>
       </c>
-      <c r="B3" s="5"/>
-      <c r="C3" s="5"/>
-      <c r="D3" s="6"/>
-    </row>
-    <row r="4" spans="1:20" ht="16.8" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A4" s="7" t="s">
+      <c r="B3" s="24"/>
+      <c r="C3" s="24"/>
+      <c r="D3" s="25"/>
+    </row>
+    <row r="4" spans="1:20" ht="17" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A4" s="3" t="s">
         <v>2</v>
       </c>
-      <c r="B4" s="8" t="s">
+      <c r="B4" s="4" t="s">
         <v>3</v>
       </c>
-      <c r="C4" s="8" t="s">
+      <c r="C4" s="4" t="s">
         <v>4</v>
       </c>
-      <c r="D4" s="9" t="s">
+      <c r="D4" s="5" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="5" spans="1:20" x14ac:dyDescent="0.3">
-      <c r="A5" s="10" t="s">
+    <row r="5" spans="1:20" x14ac:dyDescent="0.2">
+      <c r="A5" s="6" t="s">
         <v>6</v>
       </c>
-      <c r="B5" s="11"/>
-      <c r="C5" s="11"/>
-      <c r="D5" s="12"/>
-    </row>
-    <row r="6" spans="1:20" x14ac:dyDescent="0.3">
-      <c r="A6" s="13" t="s">
+      <c r="B5" s="7"/>
+      <c r="C5" s="7"/>
+      <c r="D5" s="8"/>
+    </row>
+    <row r="6" spans="1:20" x14ac:dyDescent="0.2">
+      <c r="A6" s="9" t="s">
         <v>7</v>
       </c>
-      <c r="B6" s="14">
+      <c r="B6" s="10">
         <v>16370</v>
       </c>
-      <c r="C6" s="14">
+      <c r="C6" s="10">
         <v>15507</v>
       </c>
-      <c r="D6" s="15">
+      <c r="D6" s="11">
         <v>0.94728161270616984</v>
       </c>
     </row>
-    <row r="7" spans="1:20" x14ac:dyDescent="0.3">
-      <c r="A7" s="13" t="s">
+    <row r="7" spans="1:20" x14ac:dyDescent="0.2">
+      <c r="A7" s="9" t="s">
         <v>8</v>
       </c>
-      <c r="B7" s="14">
+      <c r="B7" s="10">
         <v>8881</v>
       </c>
-      <c r="C7" s="14">
+      <c r="C7" s="10">
         <v>7956</v>
       </c>
-      <c r="D7" s="15">
+      <c r="D7" s="11">
         <v>0.89584506249296247</v>
       </c>
     </row>
-    <row r="8" spans="1:20" x14ac:dyDescent="0.3">
-      <c r="A8" s="13" t="s">
+    <row r="8" spans="1:20" x14ac:dyDescent="0.2">
+      <c r="A8" s="9" t="s">
         <v>9</v>
       </c>
-      <c r="B8" s="14">
+      <c r="B8" s="10">
         <v>37906</v>
       </c>
-      <c r="C8" s="14">
+      <c r="C8" s="10">
         <v>34900</v>
       </c>
-      <c r="D8" s="15">
+      <c r="D8" s="11">
         <v>0.92069857014720624</v>
       </c>
     </row>
-    <row r="9" spans="1:20" x14ac:dyDescent="0.3">
-      <c r="A9" s="13" t="s">
+    <row r="9" spans="1:20" x14ac:dyDescent="0.2">
+      <c r="A9" s="9" t="s">
         <v>10</v>
       </c>
-      <c r="B9" s="14">
+      <c r="B9" s="10">
         <v>10341</v>
       </c>
-      <c r="C9" s="14">
+      <c r="C9" s="10">
         <v>9462</v>
       </c>
-      <c r="D9" s="15">
+      <c r="D9" s="11">
         <v>0.91499854946330139</v>
       </c>
     </row>
-    <row r="10" spans="1:20" x14ac:dyDescent="0.3">
-      <c r="A10" s="13" t="s">
+    <row r="10" spans="1:20" x14ac:dyDescent="0.2">
+      <c r="A10" s="9" t="s">
         <v>11</v>
       </c>
-      <c r="B10" s="14">
+      <c r="B10" s="10">
         <v>9555</v>
       </c>
-      <c r="C10" s="14">
+      <c r="C10" s="10">
         <v>8867</v>
       </c>
-      <c r="D10" s="15">
+      <c r="D10" s="11">
         <v>0.92799581371009943</v>
       </c>
     </row>
-    <row r="11" spans="1:20" x14ac:dyDescent="0.3">
-      <c r="A11" s="13" t="s">
+    <row r="11" spans="1:20" x14ac:dyDescent="0.2">
+      <c r="A11" s="9" t="s">
         <v>12</v>
       </c>
-      <c r="B11" s="14">
+      <c r="B11" s="10">
         <v>36559</v>
       </c>
-      <c r="C11" s="14">
+      <c r="C11" s="10">
         <v>33177</v>
       </c>
-      <c r="D11" s="15">
+      <c r="D11" s="11">
         <v>0.90749199923411472</v>
       </c>
     </row>
-    <row r="12" spans="1:20" x14ac:dyDescent="0.3">
-      <c r="A12" s="13" t="s">
+    <row r="12" spans="1:20" x14ac:dyDescent="0.2">
+      <c r="A12" s="9" t="s">
         <v>13</v>
       </c>
-      <c r="B12" s="14">
+      <c r="B12" s="10">
         <v>18381</v>
       </c>
-      <c r="C12" s="14">
+      <c r="C12" s="10">
         <v>12552</v>
       </c>
-      <c r="D12" s="15">
+      <c r="D12" s="11">
         <v>0.68287905989880859</v>
       </c>
     </row>
-    <row r="13" spans="1:20" x14ac:dyDescent="0.3">
-      <c r="A13" s="13" t="s">
+    <row r="13" spans="1:20" x14ac:dyDescent="0.2">
+      <c r="A13" s="9" t="s">
         <v>14</v>
       </c>
-      <c r="B13" s="14">
+      <c r="B13" s="10">
         <v>21917</v>
       </c>
-      <c r="C13" s="14">
+      <c r="C13" s="10">
         <v>14502</v>
       </c>
-      <c r="D13" s="15">
+      <c r="D13" s="11">
         <v>0.66167814938175851</v>
       </c>
     </row>
-    <row r="14" spans="1:20" x14ac:dyDescent="0.3">
-      <c r="A14" s="13" t="s">
+    <row r="14" spans="1:20" x14ac:dyDescent="0.2">
+      <c r="A14" s="9" t="s">
         <v>15</v>
       </c>
-      <c r="B14" s="14">
+      <c r="B14" s="10">
         <v>11458</v>
       </c>
-      <c r="C14" s="14">
+      <c r="C14" s="10">
         <v>10516</v>
       </c>
-      <c r="D14" s="15">
+      <c r="D14" s="11">
         <v>0.91778669924943268</v>
       </c>
     </row>
-    <row r="15" spans="1:20" x14ac:dyDescent="0.3">
-      <c r="A15" s="13" t="s">
+    <row r="15" spans="1:20" x14ac:dyDescent="0.2">
+      <c r="A15" s="9" t="s">
         <v>16</v>
       </c>
-      <c r="B15" s="14">
+      <c r="B15" s="10">
         <v>40097</v>
       </c>
-      <c r="C15" s="14">
+      <c r="C15" s="10">
         <v>36966</v>
       </c>
-      <c r="D15" s="15">
+      <c r="D15" s="11">
         <v>0.92191435768261965</v>
       </c>
     </row>
-    <row r="16" spans="1:20" x14ac:dyDescent="0.3">
-      <c r="A16" s="13" t="s">
+    <row r="16" spans="1:20" x14ac:dyDescent="0.2">
+      <c r="A16" s="9" t="s">
         <v>17</v>
       </c>
-      <c r="B16" s="14">
+      <c r="B16" s="10">
         <v>24775</v>
       </c>
-      <c r="C16" s="14">
+      <c r="C16" s="10">
         <v>21911</v>
       </c>
-      <c r="D16" s="15">
+      <c r="D16" s="11">
         <v>0.88439959636730581</v>
       </c>
     </row>
-    <row r="17" spans="1:19" x14ac:dyDescent="0.3">
-      <c r="A17" s="13" t="s">
+    <row r="17" spans="1:19" x14ac:dyDescent="0.2">
+      <c r="A17" s="9" t="s">
         <v>18</v>
       </c>
-      <c r="B17" s="14">
+      <c r="B17" s="10">
         <v>518</v>
       </c>
-      <c r="C17" s="14">
+      <c r="C17" s="10">
         <v>154</v>
       </c>
-      <c r="D17" s="15">
+      <c r="D17" s="11">
         <v>0.29729729729729731</v>
       </c>
     </row>
-    <row r="18" spans="1:19" x14ac:dyDescent="0.3">
-      <c r="A18" s="13" t="s">
+    <row r="18" spans="1:19" x14ac:dyDescent="0.2">
+      <c r="A18" s="9" t="s">
         <v>19</v>
       </c>
-      <c r="B18" s="14" t="s">
+      <c r="B18" s="10" t="s">
         <v>20</v>
       </c>
-      <c r="C18" s="14" t="s">
+      <c r="C18" s="10" t="s">
         <v>20</v>
       </c>
-      <c r="D18" s="15" t="s">
+      <c r="D18" s="11" t="s">
         <v>20</v>
       </c>
     </row>
-    <row r="19" spans="1:19" x14ac:dyDescent="0.3">
-      <c r="A19" s="13" t="s">
+    <row r="19" spans="1:19" x14ac:dyDescent="0.2">
+      <c r="A19" s="9" t="s">
         <v>21</v>
       </c>
-      <c r="B19" s="14">
+      <c r="B19" s="10">
         <v>86</v>
       </c>
-      <c r="C19" s="14">
+      <c r="C19" s="10">
         <v>37</v>
       </c>
-      <c r="D19" s="15">
+      <c r="D19" s="11">
         <v>0.43023255813953487</v>
       </c>
     </row>
-    <row r="20" spans="1:19" x14ac:dyDescent="0.3">
-      <c r="A20" s="16" t="s">
+    <row r="20" spans="1:19" x14ac:dyDescent="0.2">
+      <c r="A20" s="12" t="s">
         <v>22</v>
       </c>
-      <c r="B20" s="14">
+      <c r="B20" s="10">
         <v>5</v>
       </c>
-      <c r="C20" s="14">
+      <c r="C20" s="10">
         <v>2</v>
       </c>
-      <c r="D20" s="15">
+      <c r="D20" s="11">
         <v>0.4</v>
       </c>
     </row>
-    <row r="21" spans="1:19" x14ac:dyDescent="0.3">
-      <c r="A21" s="16" t="s">
+    <row r="21" spans="1:19" x14ac:dyDescent="0.2">
+      <c r="A21" s="12" t="s">
         <v>23</v>
       </c>
-      <c r="B21" s="14">
+      <c r="B21" s="10">
         <v>26919</v>
       </c>
-      <c r="C21" s="14">
+      <c r="C21" s="10">
         <v>22885</v>
       </c>
-      <c r="D21" s="15">
+      <c r="D21" s="11">
         <v>0.85014302165756528</v>
       </c>
     </row>
-    <row r="22" spans="1:19" x14ac:dyDescent="0.3">
-      <c r="A22" s="16" t="s">
+    <row r="22" spans="1:19" x14ac:dyDescent="0.2">
+      <c r="A22" s="12" t="s">
         <v>24</v>
       </c>
-      <c r="B22" s="17">
+      <c r="B22" s="13">
         <v>5422</v>
       </c>
-      <c r="C22" s="17">
+      <c r="C22" s="13">
         <v>891</v>
       </c>
-      <c r="D22" s="18">
+      <c r="D22" s="14">
         <v>0.16433050534857985</v>
       </c>
     </row>
-    <row r="23" spans="1:19" ht="16.8" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A23" s="19" t="s">
+    <row r="23" spans="1:19" ht="17" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A23" s="15" t="s">
         <v>25</v>
       </c>
-      <c r="B23" s="20">
+      <c r="B23" s="16">
         <v>269190</v>
       </c>
-      <c r="C23" s="20">
+      <c r="C23" s="16">
         <v>230285</v>
       </c>
-      <c r="D23" s="21">
+      <c r="D23" s="17">
         <v>0.85547382889408963</v>
       </c>
     </row>
-    <row r="24" spans="1:19" ht="13.65" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.35"/>
-    <row r="25" spans="1:19" ht="12.75" customHeight="1" thickTop="1" x14ac:dyDescent="0.3">
-      <c r="A25" s="4" t="s">
+    <row r="24" spans="1:19" ht="13.75" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.25"/>
+    <row r="25" spans="1:19" ht="12.75" customHeight="1" thickTop="1" x14ac:dyDescent="0.2">
+      <c r="A25" s="23" t="s">
         <v>26</v>
       </c>
-      <c r="B25" s="5"/>
-      <c r="C25" s="5"/>
-      <c r="D25" s="6"/>
-    </row>
-    <row r="26" spans="1:19" ht="12.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A26" s="7" t="s">
+      <c r="B25" s="24"/>
+      <c r="C25" s="24"/>
+      <c r="D25" s="25"/>
+    </row>
+    <row r="26" spans="1:19" ht="12.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A26" s="3" t="s">
         <v>2</v>
       </c>
-      <c r="B26" s="8" t="s">
+      <c r="B26" s="4" t="s">
         <v>3</v>
       </c>
-      <c r="C26" s="8" t="s">
+      <c r="C26" s="4" t="s">
         <v>4</v>
       </c>
-      <c r="D26" s="9" t="s">
+      <c r="D26" s="5" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="27" spans="1:19" ht="12.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A27" s="10" t="s">
+    <row r="27" spans="1:19" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A27" s="6" t="s">
         <v>6</v>
       </c>
-      <c r="B27" s="11"/>
-      <c r="C27" s="11"/>
-      <c r="D27" s="22"/>
-    </row>
-    <row r="28" spans="1:19" ht="12.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A28" s="13" t="s">
+      <c r="B27" s="7"/>
+      <c r="C27" s="7"/>
+      <c r="D27" s="18"/>
+    </row>
+    <row r="28" spans="1:19" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A28" s="9" t="s">
         <v>7</v>
       </c>
-      <c r="B28" s="14">
+      <c r="B28" s="10">
         <v>14012</v>
       </c>
-      <c r="C28" s="14">
+      <c r="C28" s="10">
         <v>13618</v>
       </c>
-      <c r="D28" s="15">
+      <c r="D28" s="11">
         <v>0.97188124464744508</v>
       </c>
     </row>
-    <row r="29" spans="1:19" ht="12.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A29" s="13" t="s">
+    <row r="29" spans="1:19" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A29" s="9" t="s">
         <v>8</v>
       </c>
-      <c r="B29" s="14">
+      <c r="B29" s="10">
         <v>6706</v>
       </c>
-      <c r="C29" s="14">
+      <c r="C29" s="10">
         <v>6469</v>
       </c>
-      <c r="D29" s="15">
+      <c r="D29" s="11">
         <v>0.96465851476289888</v>
       </c>
-      <c r="Q29" s="23"/>
-      <c r="R29" s="23"/>
-      <c r="S29" s="23"/>
-    </row>
-    <row r="30" spans="1:19" ht="12.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A30" s="13" t="s">
+      <c r="Q29" s="19"/>
+      <c r="R29" s="19"/>
+      <c r="S29" s="19"/>
+    </row>
+    <row r="30" spans="1:19" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A30" s="9" t="s">
         <v>9</v>
       </c>
-      <c r="B30" s="14">
+      <c r="B30" s="10">
         <v>28089</v>
       </c>
-      <c r="C30" s="14">
+      <c r="C30" s="10">
         <v>27240</v>
       </c>
-      <c r="D30" s="15">
+      <c r="D30" s="11">
         <v>0.96977464487877818</v>
       </c>
-      <c r="Q30" s="23"/>
-      <c r="R30" s="23"/>
-      <c r="S30" s="23"/>
-    </row>
-    <row r="31" spans="1:19" ht="12.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A31" s="13" t="s">
+      <c r="Q30" s="19"/>
+      <c r="R30" s="19"/>
+      <c r="S30" s="19"/>
+    </row>
+    <row r="31" spans="1:19" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A31" s="9" t="s">
         <v>10</v>
       </c>
-      <c r="B31" s="14">
+      <c r="B31" s="10">
         <v>8440</v>
       </c>
-      <c r="C31" s="14">
+      <c r="C31" s="10">
         <v>8223</v>
       </c>
-      <c r="D31" s="15">
+      <c r="D31" s="11">
         <v>0.97428909952606635</v>
       </c>
-      <c r="Q31" s="23"/>
-      <c r="R31" s="23"/>
-      <c r="S31" s="23"/>
-    </row>
-    <row r="32" spans="1:19" ht="12.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A32" s="13" t="s">
+      <c r="Q31" s="19"/>
+      <c r="R31" s="19"/>
+      <c r="S31" s="19"/>
+    </row>
+    <row r="32" spans="1:19" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A32" s="9" t="s">
         <v>11</v>
       </c>
-      <c r="B32" s="14">
+      <c r="B32" s="10">
         <v>9305</v>
       </c>
-      <c r="C32" s="14">
+      <c r="C32" s="10">
         <v>9077</v>
       </c>
-      <c r="D32" s="15">
+      <c r="D32" s="11">
         <v>0.97549704459967757</v>
       </c>
-      <c r="Q32" s="23"/>
-      <c r="R32" s="23"/>
-      <c r="S32" s="23"/>
-    </row>
-    <row r="33" spans="1:4" ht="12.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A33" s="13" t="s">
+      <c r="Q32" s="19"/>
+      <c r="R32" s="19"/>
+      <c r="S32" s="19"/>
+    </row>
+    <row r="33" spans="1:4" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A33" s="9" t="s">
         <v>12</v>
       </c>
-      <c r="B33" s="14">
+      <c r="B33" s="10">
         <v>26333</v>
       </c>
-      <c r="C33" s="14">
+      <c r="C33" s="10">
         <v>25556</v>
       </c>
-      <c r="D33" s="15">
+      <c r="D33" s="11">
         <v>0.9704932973835112</v>
       </c>
     </row>
-    <row r="34" spans="1:4" ht="12.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A34" s="13" t="s">
+    <row r="34" spans="1:4" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A34" s="9" t="s">
         <v>13</v>
       </c>
-      <c r="B34" s="14">
+      <c r="B34" s="10">
         <v>8689</v>
       </c>
-      <c r="C34" s="14">
+      <c r="C34" s="10">
         <v>8010</v>
       </c>
-      <c r="D34" s="15">
+      <c r="D34" s="11">
         <v>0.92185521924272074</v>
       </c>
     </row>
-    <row r="35" spans="1:4" ht="12.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A35" s="13" t="s">
+    <row r="35" spans="1:4" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A35" s="9" t="s">
         <v>14</v>
       </c>
-      <c r="B35" s="14">
+      <c r="B35" s="10">
         <v>10075</v>
       </c>
-      <c r="C35" s="14">
+      <c r="C35" s="10">
         <v>9410</v>
       </c>
-      <c r="D35" s="15">
+      <c r="D35" s="11">
         <v>0.93399503722084365</v>
       </c>
     </row>
-    <row r="36" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A36" s="13" t="s">
+    <row r="36" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A36" s="9" t="s">
         <v>15</v>
       </c>
-      <c r="B36" s="14">
+      <c r="B36" s="10">
         <v>8874</v>
       </c>
-      <c r="C36" s="14">
+      <c r="C36" s="10">
         <v>8612</v>
       </c>
-      <c r="D36" s="15">
+      <c r="D36" s="11">
         <v>0.97047554654045531</v>
       </c>
     </row>
-    <row r="37" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A37" s="13" t="s">
+    <row r="37" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A37" s="9" t="s">
         <v>16</v>
       </c>
-      <c r="B37" s="14">
+      <c r="B37" s="10">
         <v>32543</v>
       </c>
-      <c r="C37" s="14">
+      <c r="C37" s="10">
         <v>31556</v>
       </c>
-      <c r="D37" s="15">
+      <c r="D37" s="11">
         <v>0.96967089696708975</v>
       </c>
     </row>
-    <row r="38" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A38" s="13" t="s">
+    <row r="38" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A38" s="9" t="s">
         <v>17</v>
       </c>
-      <c r="B38" s="14">
+      <c r="B38" s="10">
         <v>8315</v>
       </c>
-      <c r="C38" s="14">
+      <c r="C38" s="10">
         <v>7937</v>
       </c>
-      <c r="D38" s="15">
+      <c r="D38" s="11">
         <v>0.95453998797354178</v>
       </c>
     </row>
-    <row r="39" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A39" s="13" t="s">
+    <row r="39" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A39" s="9" t="s">
         <v>18</v>
       </c>
-      <c r="B39" s="14">
+      <c r="B39" s="10">
         <v>1</v>
       </c>
-      <c r="C39" s="14">
+      <c r="C39" s="10">
         <v>1</v>
       </c>
-      <c r="D39" s="15">
+      <c r="D39" s="11">
         <v>1</v>
       </c>
     </row>
-    <row r="40" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A40" s="13" t="s">
+    <row r="40" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A40" s="9" t="s">
         <v>19</v>
       </c>
-      <c r="B40" s="14" t="s">
+      <c r="B40" s="10" t="s">
         <v>20</v>
       </c>
-      <c r="C40" s="14" t="s">
+      <c r="C40" s="10" t="s">
         <v>20</v>
       </c>
-      <c r="D40" s="15" t="s">
+      <c r="D40" s="11" t="s">
         <v>20</v>
       </c>
     </row>
-    <row r="41" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A41" s="13" t="s">
+    <row r="41" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A41" s="9" t="s">
         <v>21</v>
       </c>
-      <c r="B41" s="14">
+      <c r="B41" s="10">
         <v>11</v>
       </c>
-      <c r="C41" s="14">
+      <c r="C41" s="10">
         <v>10</v>
       </c>
-      <c r="D41" s="15">
+      <c r="D41" s="11">
         <v>0.90909090909090906</v>
       </c>
     </row>
-    <row r="42" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A42" s="16" t="s">
+    <row r="42" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A42" s="12" t="s">
         <v>22</v>
       </c>
-      <c r="B42" s="14" t="s">
+      <c r="B42" s="10" t="s">
         <v>20</v>
       </c>
-      <c r="C42" s="14" t="s">
+      <c r="C42" s="10" t="s">
         <v>20</v>
       </c>
-      <c r="D42" s="15" t="s">
+      <c r="D42" s="11" t="s">
         <v>20</v>
       </c>
     </row>
-    <row r="43" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A43" s="16" t="s">
+    <row r="43" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A43" s="12" t="s">
         <v>23</v>
       </c>
-      <c r="B43" s="14">
+      <c r="B43" s="10">
         <v>23365</v>
       </c>
-      <c r="C43" s="14">
+      <c r="C43" s="10">
         <v>22435</v>
       </c>
-      <c r="D43" s="15">
+      <c r="D43" s="11">
         <v>0.96019687566873524</v>
       </c>
     </row>
-    <row r="44" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A44" s="16" t="s">
+    <row r="44" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A44" s="12" t="s">
         <v>24</v>
       </c>
-      <c r="B44" s="17">
+      <c r="B44" s="13">
         <v>59</v>
       </c>
-      <c r="C44" s="17">
+      <c r="C44" s="13">
         <v>57</v>
       </c>
-      <c r="D44" s="18">
+      <c r="D44" s="14">
         <v>0.96610169491525422</v>
       </c>
     </row>
-    <row r="45" spans="1:4" ht="16.8" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A45" s="19" t="s">
+    <row r="45" spans="1:4" ht="17" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A45" s="15" t="s">
         <v>25</v>
       </c>
-      <c r="B45" s="20">
+      <c r="B45" s="16">
         <v>184817</v>
       </c>
-      <c r="C45" s="20">
+      <c r="C45" s="16">
         <v>178211</v>
       </c>
-      <c r="D45" s="21">
+      <c r="D45" s="17">
         <v>0.96425653484257401</v>
       </c>
     </row>
-    <row r="46" spans="1:4" ht="16.8" thickTop="1" x14ac:dyDescent="0.3"/>
-    <row r="47" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A47" s="23" t="s">
+    <row r="46" spans="1:4" ht="17" thickTop="1" x14ac:dyDescent="0.2"/>
+    <row r="47" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A47" s="19" t="s">
         <v>27</v>
       </c>
     </row>
-    <row r="49" spans="1:16" x14ac:dyDescent="0.3">
-      <c r="A49" s="24" t="s">
+    <row r="49" spans="1:16" x14ac:dyDescent="0.2">
+      <c r="A49" s="20" t="s">
         <v>28</v>
       </c>
     </row>
-    <row r="50" spans="1:16" x14ac:dyDescent="0.3">
-      <c r="A50" s="24"/>
-    </row>
-    <row r="51" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="50" spans="1:16" x14ac:dyDescent="0.2">
+      <c r="A50" s="20"/>
+    </row>
+    <row r="51" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A51" t="s">
         <v>29</v>
       </c>
-      <c r="K51" s="23"/>
-      <c r="L51" s="23"/>
-      <c r="M51" s="23"/>
-      <c r="N51" s="23"/>
-      <c r="O51" s="23"/>
-      <c r="P51" s="23"/>
-    </row>
-    <row r="52" spans="1:16" x14ac:dyDescent="0.3">
-      <c r="K52" s="23"/>
-      <c r="L52" s="23"/>
-      <c r="M52" s="23"/>
-      <c r="N52" s="23"/>
-      <c r="O52" s="23"/>
-      <c r="P52" s="23"/>
-    </row>
-    <row r="53" spans="1:16" x14ac:dyDescent="0.3">
+      <c r="K51" s="19"/>
+      <c r="L51" s="19"/>
+      <c r="M51" s="19"/>
+      <c r="N51" s="19"/>
+      <c r="O51" s="19"/>
+      <c r="P51" s="19"/>
+    </row>
+    <row r="52" spans="1:16" x14ac:dyDescent="0.2">
+      <c r="K52" s="19"/>
+      <c r="L52" s="19"/>
+      <c r="M52" s="19"/>
+      <c r="N52" s="19"/>
+      <c r="O52" s="19"/>
+      <c r="P52" s="19"/>
+    </row>
+    <row r="53" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A53" t="s">
         <v>30</v>
       </c>
-      <c r="K53" s="23"/>
-      <c r="L53" s="23"/>
-      <c r="M53" s="23"/>
-      <c r="N53" s="23"/>
-      <c r="O53" s="23"/>
-      <c r="P53" s="23"/>
-    </row>
-    <row r="54" spans="1:16" x14ac:dyDescent="0.3">
-      <c r="K54" s="23"/>
-      <c r="L54" s="23"/>
-      <c r="M54" s="23"/>
-      <c r="N54" s="23"/>
-      <c r="O54" s="23"/>
-      <c r="P54" s="23"/>
-    </row>
-    <row r="55" spans="1:16" x14ac:dyDescent="0.3">
-      <c r="A55" s="25" t="s">
+      <c r="K53" s="19"/>
+      <c r="L53" s="19"/>
+      <c r="M53" s="19"/>
+      <c r="N53" s="19"/>
+      <c r="O53" s="19"/>
+      <c r="P53" s="19"/>
+    </row>
+    <row r="54" spans="1:16" x14ac:dyDescent="0.2">
+      <c r="K54" s="19"/>
+      <c r="L54" s="19"/>
+      <c r="M54" s="19"/>
+      <c r="N54" s="19"/>
+      <c r="O54" s="19"/>
+      <c r="P54" s="19"/>
+    </row>
+    <row r="55" spans="1:16" x14ac:dyDescent="0.2">
+      <c r="A55" s="26" t="s">
         <v>31</v>
       </c>
-      <c r="B55" s="26"/>
-      <c r="C55" s="26"/>
-      <c r="D55" s="26"/>
-      <c r="E55" s="26"/>
-      <c r="F55" s="26"/>
-      <c r="G55" s="26"/>
-      <c r="H55" s="26"/>
-      <c r="I55" s="26"/>
-      <c r="J55" s="26"/>
-      <c r="K55" s="26"/>
-      <c r="L55" s="26"/>
-      <c r="M55" s="26"/>
-      <c r="N55" s="26"/>
-      <c r="O55" s="26"/>
-      <c r="P55" s="26"/>
-    </row>
-    <row r="56" spans="1:16" x14ac:dyDescent="0.3">
-      <c r="A56" s="27"/>
-    </row>
-    <row r="57" spans="1:16" x14ac:dyDescent="0.3">
+      <c r="B55" s="27"/>
+      <c r="C55" s="27"/>
+      <c r="D55" s="27"/>
+      <c r="E55" s="27"/>
+      <c r="F55" s="27"/>
+      <c r="G55" s="27"/>
+      <c r="H55" s="27"/>
+      <c r="I55" s="27"/>
+      <c r="J55" s="27"/>
+      <c r="K55" s="27"/>
+      <c r="L55" s="27"/>
+      <c r="M55" s="27"/>
+      <c r="N55" s="27"/>
+      <c r="O55" s="27"/>
+      <c r="P55" s="27"/>
+    </row>
+    <row r="56" spans="1:16" x14ac:dyDescent="0.2">
+      <c r="A56" s="21"/>
+    </row>
+    <row r="57" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A57" s="28" t="s">
         <v>32</v>
       </c>
@@ -1590,13 +1590,13 @@
       <c r="I57" s="29"/>
       <c r="J57" s="29"/>
     </row>
-    <row r="58" spans="1:16" x14ac:dyDescent="0.3">
-      <c r="A58" s="23" t="s">
+    <row r="58" spans="1:16" x14ac:dyDescent="0.2">
+      <c r="A58" s="19" t="s">
         <v>33</v>
       </c>
     </row>
-    <row r="60" spans="1:16" x14ac:dyDescent="0.3">
-      <c r="A60" s="23" t="s">
+    <row r="60" spans="1:16" x14ac:dyDescent="0.2">
+      <c r="A60" s="19" t="s">
         <v>34</v>
       </c>
     </row>

</xml_diff>